<commit_message>
Se actualizan predicciones de la ultima semana pra evitar predicciones negativas y se agrega detalle del modelo en el excel
</commit_message>
<xml_diff>
--- a/data/output/forecast_results_Recursivo.xlsx
+++ b/data/output/forecast_results_Recursivo.xlsx
@@ -468,21 +468,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.25</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2983.891965293659</v>
+        <v>3274.912277742098</v>
       </c>
       <c r="D2" t="n">
-        <v>2593.49546031901</v>
+        <v>2838.845765118879</v>
       </c>
       <c r="E2" t="n">
-        <v>13.54892572862405</v>
+        <v>14.71100331193007</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[10881.681426695184, 19977.92409355593, 8181.577551900251, 26984.766215818876, 23128.171580840382, 21068.13000337964, 16262.491946078893]</t>
+          <t>[10722.697736602024, 19791.579510256546, 7896.481064513266, 26674.562956476148, 22781.427169962437, 20655.84831741571, 15708.64190945481]</t>
         </is>
       </c>
     </row>
@@ -494,21 +494,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.21-b0.05-g0.16</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>333.9701790220622</v>
+        <v>328.3938154364798</v>
       </c>
       <c r="D3" t="n">
-        <v>276.1587903363479</v>
+        <v>268.61976793651</v>
       </c>
       <c r="E3" t="n">
-        <v>20.5914346430878</v>
+        <v>20.00423459076796</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[838.2191825208924, 973.3130183977378, 805.4571059010256, 1319.1340956211905, 1299.8286278653081, 512.0124038291065, 1498.9240335103038]</t>
+          <t>[841.7592973951706, 977.8559950696409, 812.5971398487513, 1330.5484574053605, 1308.294050068608, 516.8977418798456, 1511.708942777053]</t>
         </is>
       </c>
     </row>
@@ -520,21 +520,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.17-g0.09</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>291.8582789592426</v>
+        <v>289.1029541609326</v>
       </c>
       <c r="D4" t="n">
-        <v>251.4524367018846</v>
+        <v>251.0654841691924</v>
       </c>
       <c r="E4" t="n">
-        <v>38.65857415648701</v>
+        <v>38.33089297277512</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[974.2456555427192, 1268.62556893577, 805.819650868098, 1214.541662111613, 1347.390293709309, 914.4855557315038, 1547.0903953043369]</t>
+          <t>[970.4701112430387, 1272.6144344396685, 799.0775903455095, 1215.3485033485892, 1344.5233960971711, 909.773527265567, 1559.9264875184817]</t>
         </is>
       </c>
     </row>
@@ -546,21 +546,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARIMA(1,0,2)</t>
+          <t>ARIMA(p1-d0-q2)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>336.5194193138352</v>
+        <v>334.2351657595904</v>
       </c>
       <c r="D5" t="n">
-        <v>285.7252310753487</v>
+        <v>284.5447059441424</v>
       </c>
       <c r="E5" t="n">
-        <v>42.38245245021906</v>
+        <v>42.33236976282187</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[408.49942010535744, 396.89429954446746, 399.2608021414295, 399.3088698628463, 399.3098462006053, 399.3098660316976, 399.30986643450103]</t>
+          <t>[408.04805312842296, 396.6244092106537, 398.96183922085896, 399.00846552667105, 399.0093956132979, 399.0094141663683, 399.00941453645896]</t>
         </is>
       </c>
     </row>
@@ -572,21 +572,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARIMA(2,2,2)</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.07-b0.09-g0.07</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>283.3502531477282</v>
+        <v>227.3766104095246</v>
       </c>
       <c r="D6" t="n">
-        <v>226.1416547625496</v>
+        <v>193.2775777522199</v>
       </c>
       <c r="E6" t="n">
-        <v>80.63938762591782</v>
+        <v>47.60336434187578</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[571.0156782172999, 543.1084049644135, 550.7669881415657, 550.1571644771163, 551.1100132388092, 551.6753015248588, 552.3076117943649]</t>
+          <t>[316.80331104077624, 508.7905501535252, 219.51133679102156, 371.3828815070573, 581.1229156093686, 587.9257368227724, 570.9783195370366]</t>
         </is>
       </c>
     </row>
@@ -598,21 +598,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2687.287703914498</v>
+        <v>1759.673900235364</v>
       </c>
       <c r="D7" t="n">
-        <v>2074.185785629995</v>
+        <v>1351.032855740508</v>
       </c>
       <c r="E7" t="n">
-        <v>93.74375590696874</v>
+        <v>105.2191632676511</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[2132.577267715805, 366.5453739035434, -709.7878134121343, -581.0106112802156, 1213.260512929439, 50.16228189967501, -575.7753375878913]</t>
+          <t>[3070.443105642922, 1479.973361908491, 630.7804663095528, 999.0053479070252, 3002.1675989295945, 2035.0564440385149, 1585.652428417881]</t>
         </is>
       </c>
     </row>
@@ -624,21 +624,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.22-g0.11</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>288.0451124246934</v>
+        <v>283.9996866413552</v>
       </c>
       <c r="D8" t="n">
-        <v>254.4773949664183</v>
+        <v>250.3600261068594</v>
       </c>
       <c r="E8" t="n">
-        <v>28.17248637795949</v>
+        <v>27.59347678905311</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[372.1586408865526, 378.971661655654, 948.3268182635245, 1557.3005627644493, 459.0476075123164, 1268.0219976378353, 547.5285783174595]</t>
+          <t>[380.30851972400274, 386.8808168365863, 947.9508258629836, 1559.4739893367773, 464.1664832916673, 1268.2855123793224, 552.8863463052567]</t>
         </is>
       </c>
     </row>
@@ -650,21 +650,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.35-b0.14-g0.05</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>908.4937516852513</v>
+        <v>972.9309441467058</v>
       </c>
       <c r="D9" t="n">
-        <v>687.1432888352144</v>
+        <v>696.832413603094</v>
       </c>
       <c r="E9" t="n">
-        <v>128.2959434012298</v>
+        <v>34.65323107458707</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[4105.224206340649, 4165.531329003082, -485.81025287686043, 4085.3170210412636, 3477.2091345726144, 3300.915780337051, 3666.8964283300074]</t>
+          <t>[4351.614056268247, 4316.351852039614, 0.0, 4570.698566725058, 4057.5515017456037, 3932.3826945113487, 4360.477445735099]</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.17-g0.05</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4697.803164801273</v>
+        <v>4692.596174553106</v>
       </c>
       <c r="D10" t="n">
-        <v>3972.227872268404</v>
+        <v>3966.583286869793</v>
       </c>
       <c r="E10" t="n">
-        <v>51.05546963779133</v>
+        <v>50.98926954552029</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[16734.568642106573, 13120.236273571863, 12777.125970244295, 13435.334899806914, 21872.237737447205, 12939.07184579125, 14152.271677399316]</t>
+          <t>[16727.34202541427, 13113.505666532103, 12771.113541106766, 13427.067535160699, 21865.395893661705, 12930.766479015061, 14144.118949411484]</t>
         </is>
       </c>
     </row>
@@ -702,21 +702,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARIMA(2,0,2)</t>
+          <t>ARIMA(p2-d0-q2)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>696.913528150028</v>
+        <v>696.8842539251059</v>
       </c>
       <c r="D11" t="n">
-        <v>539.2331587530701</v>
+        <v>539.1375945793428</v>
       </c>
       <c r="E11" t="n">
-        <v>28.82065771577534</v>
+        <v>28.81453344400591</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[2130.7054902247464, 1712.7290428221768, 1786.4600308253825, 2197.7575170872783, 2385.5745286661368, 2140.6227184053014, 1825.8250220424177]</t>
+          <t>[2130.4072473481165, 1712.6578091970082, 1786.6187246339282, 2197.863764547104, 2385.452589159144, 2140.4053598104156, 1825.7434424340522]</t>
         </is>
       </c>
     </row>
@@ -728,21 +728,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.89-g0.1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3193.888522511484</v>
+        <v>3140.372051758121</v>
       </c>
       <c r="D12" t="n">
-        <v>2576.635074365394</v>
+        <v>2531.199324910177</v>
       </c>
       <c r="E12" t="n">
-        <v>73.03095318596266</v>
+        <v>59.8024405171362</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[3198.680971888628, -129.8680104197449, 221.40544476933337, 1268.1225353185205, 2334.2350808754372, 1120.362584092571, 256.39590751636075]</t>
+          <t>[3110.0871807562967, 123.60083887450173, 389.32404120937144, 1335.8989020167262, 2383.6359294397926, 863.228672781997, 386.96357990991146]</t>
         </is>
       </c>
     </row>
@@ -754,21 +754,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ARIMA(2,1,2)</t>
+          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.2-g0.06</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1736.7280099807</v>
+        <v>1764.545580269533</v>
       </c>
       <c r="D13" t="n">
-        <v>1589.895725098084</v>
+        <v>1555.770178221579</v>
       </c>
       <c r="E13" t="n">
-        <v>38.15562761867723</v>
+        <v>36.27568395522115</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[4580.6462003863235, 4081.0193190543273, 4728.116277252031, 4216.2384353249345, 4596.324222086039, 4317.192337811957, 4521.773747806207]</t>
+          <t>[4085.813868970178, 4836.602677047438, 3246.781715432305, 5096.28263310396, 4387.652822297589, 4136.205207832191, 4332.014111975152]</t>
         </is>
       </c>
     </row>
@@ -780,21 +780,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.59-b0.58-g0.11</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11693.70434732924</v>
+        <v>13968.04175366843</v>
       </c>
       <c r="D14" t="n">
-        <v>11116.67608536774</v>
+        <v>13267.11480956027</v>
       </c>
       <c r="E14" t="n">
-        <v>187.3659804668514</v>
+        <v>221.126247476913</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[16369.225195919716, 10181.496222167665, 15148.403694740495, 21711.58520934914, 24567.333751898186, 24524.95239399824, 25517.035776398006]</t>
+          <t>[16788.9469237623, 11673.282111239849, 16986.195767990957, 23660.922577368183, 27237.406519528187, 27377.365474430375, 29362.43618662148]</t>
         </is>
       </c>
     </row>
@@ -806,21 +806,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.07-g0.05</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>881.838282644692</v>
+        <v>867.7926320885475</v>
       </c>
       <c r="D15" t="n">
-        <v>722.2445948838495</v>
+        <v>712.2549009247856</v>
       </c>
       <c r="E15" t="n">
-        <v>42.01680844929326</v>
+        <v>40.99804679444166</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[3234.733783873206, 4331.177234856745, 2339.916059493091, 4748.164363447763, 7699.848507589872, 2604.3874912513756, 4199.958903921477]</t>
+          <t>[3209.198959459306, 4301.560199203248, 2307.3166967923753, 4711.068977380947, 7662.202732024307, 2559.5007251821053, 4149.314142245404]</t>
         </is>
       </c>
     </row>
@@ -832,21 +832,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.27-g0.18</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1037.450034423125</v>
+        <v>1140.10324257694</v>
       </c>
       <c r="D16" t="n">
-        <v>841.2052833325175</v>
+        <v>881.9417432577741</v>
       </c>
       <c r="E16" t="n">
-        <v>41.50238226402676</v>
+        <v>35.39788847152437</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[3854.9312467401687, 2156.130666801082, 1041.4367352544168, 4751.085625915877, 5856.580682552267, 4301.685574997821, 2966.6160411651763]</t>
+          <t>[3739.0456511104962, 1988.913194014515, 886.6141695131505, 4433.391321402636, 5448.024008105365, 3875.8068058239096, 2531.110315229623]</t>
         </is>
       </c>
     </row>
@@ -858,21 +858,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.15-b0.05-g0.11</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1132.173622022179</v>
+        <v>1123.967082483953</v>
       </c>
       <c r="D17" t="n">
-        <v>976.0646127415469</v>
+        <v>974.5290236410672</v>
       </c>
       <c r="E17" t="n">
-        <v>20.37304847487222</v>
+        <v>20.40103770904746</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[4578.297228900191, 5231.514559081469, 3425.773930047723, 6407.9503894103555, 5973.13431353757, 2635.372168210517, 6076.727215121476]</t>
+          <t>[4599.7134224892925, 5213.823561728259, 3438.5872082901587, 6328.848437661972, 5955.0096999403995, 2672.001496008873, 6036.8344157721]</t>
         </is>
       </c>
     </row>
@@ -884,21 +884,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.33-g0.18</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1955.044620433532</v>
+        <v>1964.070233266426</v>
       </c>
       <c r="D18" t="n">
-        <v>1714.682609910396</v>
+        <v>1732.536029364453</v>
       </c>
       <c r="E18" t="n">
-        <v>43.86157984184585</v>
+        <v>44.5439851533932</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[2633.963968594873, 3544.0146161230346, 1476.5615506996003, 4039.897494306736, 3354.957125769927, 1889.3801132754115, 5734.864974401789]</t>
+          <t>[2631.908713553468, 3563.998243748816, 1441.838492994898, 4061.58255038985, 3342.2907138660407, 1907.604308015565, 5837.949184981741]</t>
         </is>
       </c>
     </row>
@@ -910,21 +910,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.09-b0.05-g0.64</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>717.8826669329251</v>
+        <v>663.5484795499465</v>
       </c>
       <c r="D19" t="n">
-        <v>592.6123351631666</v>
+        <v>603.9988448034521</v>
       </c>
       <c r="E19" t="n">
-        <v>25.32240669318101</v>
+        <v>26.73173758668018</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[2354.255195673186, 2132.4024187288724, 1402.3049295956112, 2077.4013633696914, 3107.1309379087397, 2306.016276232932, 2111.434004114124]</t>
+          <t>[2773.2443579141495, 1823.0179671124645, 851.5299106555732, 1926.0854804303656, 2588.1587316405617, 1491.5651878651302, 2267.2818500317426]</t>
         </is>
       </c>
     </row>
@@ -936,21 +936,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ARIMA(1,1,2)</t>
+          <t>ARIMA(p1-d1-q2)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>868.6641798748084</v>
+        <v>868.6114108230386</v>
       </c>
       <c r="D20" t="n">
-        <v>591.2549507676457</v>
+        <v>591.3883362650914</v>
       </c>
       <c r="E20" t="n">
-        <v>21.27693786446188</v>
+        <v>21.28754433742413</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[1788.449879791553, 2163.3224597306084, 1849.7833991980872, 2112.02381831756, 1892.6889855118602, 2076.1380855530983, 1922.703394512699]</t>
+          <t>[1788.608156757438, 2164.1339785426662, 1850.0780813180475, 2112.726082759529, 1893.0710045685723, 2076.770682884324, 1923.1408551961426]</t>
         </is>
       </c>
     </row>
@@ -962,21 +962,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ARIMA(2,0,1)</t>
+          <t>ARIMA(p2-d0-q1)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5310.04618330443</v>
+        <v>5310.230094546409</v>
       </c>
       <c r="D21" t="n">
-        <v>4803.033877682924</v>
+        <v>4803.300223307759</v>
       </c>
       <c r="E21" t="n">
-        <v>47.62167012883972</v>
+        <v>47.62148498167227</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[14746.148135692287, 13474.629776538623, 14330.240743896473, 13623.586048612919, 14199.858391382026, 13729.575025992815, 14113.347454732462]</t>
+          <t>[14746.667513740473, 13473.321197925474, 14330.255275632104, 13622.459707747772, 14199.697357898247, 13728.597242941441, 14113.059794411785]</t>
         </is>
       </c>
     </row>
@@ -988,21 +988,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ARIMA(2,2,2)</t>
+          <t>ARIMA(p2-d0-q1)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>954.0079872145378</v>
+        <v>1195.514625927227</v>
       </c>
       <c r="D22" t="n">
-        <v>704.5938474466777</v>
+        <v>969.6777239848846</v>
       </c>
       <c r="E22" t="n">
-        <v>19.49804257205312</v>
+        <v>26.00803429028172</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[5032.160375857702, 4949.346794937574, 5026.643368515835, 5027.759243694101, 5019.224533391269, 5017.084935173118, 5015.456167945348]</t>
+          <t>[5332.27117703632, 5327.400737722096, 5357.788460891841, 5331.738873047246, 5353.041827069288, 5335.667609829102, 5349.835382298299]</t>
         </is>
       </c>
     </row>
@@ -1014,21 +1014,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.56-g0.14</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2404.928022447044</v>
+        <v>2251.703215383586</v>
       </c>
       <c r="D23" t="n">
-        <v>1571.938378301484</v>
+        <v>1508.831995299819</v>
       </c>
       <c r="E23" t="n">
-        <v>9.665243321164544</v>
+        <v>9.271439447426545</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[12492.979559520709, 17288.165395543085, 9596.577196601875, 15424.924487174509, 12481.060485895996, 15194.119215564693, 14547.56749818293]</t>
+          <t>[12218.27778572724, 17132.901454933748, 9528.150872531129, 15421.173530997405, 12246.892034079157, 15673.620483486126, 14552.364249658005]</t>
         </is>
       </c>
     </row>
@@ -1040,21 +1040,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>686.0704805178635</v>
+        <v>677.5235599918963</v>
       </c>
       <c r="D24" t="n">
-        <v>538.6167328288166</v>
+        <v>528.409511341451</v>
       </c>
       <c r="E24" t="n">
-        <v>16.28773837513467</v>
+        <v>15.90141872334303</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[2546.279220853988, 3276.150615710352, 1455.6191640584427, 3108.3952872726873, 2223.120391614769, 2023.6364713592304, 2446.4817193288145]</t>
+          <t>[2556.432099540607, 3284.706231707938, 1467.3869010185547, 3114.400536906187, 2242.1599360691584, 2032.6654823399995, 2453.3822330273983]</t>
         </is>
       </c>
     </row>
@@ -1066,21 +1066,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ARIMA(0,0,1)</t>
+          <t>ARIMA(p0-d0-q1)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4719.583186022256</v>
+        <v>4719.545953910282</v>
       </c>
       <c r="D25" t="n">
-        <v>4067.342174497215</v>
+        <v>4067.596709901987</v>
       </c>
       <c r="E25" t="n">
-        <v>80.83600422664088</v>
+        <v>80.83291223834603</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[9924.270775500732, 9902.167001509382, 9902.167001509382, 9902.167001509382, 9902.167001509382, 9902.167001509382, 9902.167001509382]</t>
+          <t>[9923.919683805083, 9901.451673440502, 9901.451673440502, 9901.451673440502, 9901.451673440502, 9901.451673440502, 9901.451673440502]</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.84-b0.21-g0.66</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1068.042412906589</v>
+        <v>1485.24487402689</v>
       </c>
       <c r="D26" t="n">
-        <v>888.0522609931243</v>
+        <v>1144.990825185982</v>
       </c>
       <c r="E26" t="n">
-        <v>102.3480484795531</v>
+        <v>152.9945412176032</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[1300.3090756004672, 417.852180731311, 262.06501277949735, 700.9155737331162, 2125.0445841705186, 1212.3469027782387, 846.5786690055744]</t>
+          <t>[1632.7646932745604, 0.0, 0.0, 0.0, 1391.4992793140732, 793.2263539468155, 0.0]</t>
         </is>
       </c>
     </row>
@@ -1118,21 +1118,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.08</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>978.0010009006696</v>
+        <v>954.6250362162758</v>
       </c>
       <c r="D27" t="n">
-        <v>805.5284014921801</v>
+        <v>793.161888273081</v>
       </c>
       <c r="E27" t="n">
-        <v>273.8431316636076</v>
+        <v>266.847914863758</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[1532.3265602997972, 1548.5170312512773, 1497.4153026934737, 2019.0198590435416, 1580.831903464005, 1867.1593099650559, 1644.2659358714761]</t>
+          <t>[1509.1085700966512, 1532.0610623723921, 1409.4255378264445, 2022.161315320735, 1582.1885695108645, 1834.2152136776945, 1615.5037847598087]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se corrige grafica, estaba graficanado hasta una semana antes
</commit_message>
<xml_diff>
--- a/data/output/forecast_results_Recursivo.xlsx
+++ b/data/output/forecast_results_Recursivo.xlsx
@@ -468,21 +468,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.25</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.18-g0.26</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3274.912277742098</v>
+        <v>3370.788768434009</v>
       </c>
       <c r="D2" t="n">
-        <v>2838.845765118879</v>
+        <v>2923.907244363023</v>
       </c>
       <c r="E2" t="n">
-        <v>14.71100331193007</v>
+        <v>15.16066528805687</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[10722.697736602024, 19791.579510256546, 7896.481064513266, 26674.562956476148, 22781.427169962437, 20655.84831741571, 15708.64190945481]</t>
+          <t>[10683.529669664322, 19784.371822121757, 7812.168389276536, 26610.927829068503, 22717.963679664594, 20548.27107161089, 15464.16047229575]</t>
         </is>
       </c>
     </row>
@@ -494,21 +494,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.21-b0.05-g0.16</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.22-b0.05-g0.16</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>328.3938154364798</v>
+        <v>323.7320023642358</v>
       </c>
       <c r="D3" t="n">
-        <v>268.61976793651</v>
+        <v>262.7652561352002</v>
       </c>
       <c r="E3" t="n">
-        <v>20.00423459076796</v>
+        <v>19.4951036182859</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[841.7592973951706, 977.8559950696409, 812.5971398487513, 1330.5484574053605, 1308.294050068608, 516.8977418798456, 1511.708942777053]</t>
+          <t>[847.1671447417566, 984.1953725153573, 819.1050615010266, 1335.8387595620368, 1313.4296510772233, 523.171735963137, 1517.7354816930613]</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>289.1029541609326</v>
+        <v>288.9019799464968</v>
       </c>
       <c r="D4" t="n">
-        <v>251.0654841691924</v>
+        <v>251.1698401096004</v>
       </c>
       <c r="E4" t="n">
-        <v>38.33089297277512</v>
+        <v>38.32085397048436</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[970.4701112430387, 1272.6144344396685, 799.0775903455095, 1215.3485033485892, 1344.5233960971711, 909.773527265567, 1559.9264875184817]</t>
+          <t>[970.3712015611587, 1273.5660968454304, 798.532803654837, 1215.834807565322, 1344.5340265228135, 909.5672696464571, 1561.982921707672]</t>
         </is>
       </c>
     </row>
@@ -572,21 +572,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.07-b0.09-g0.07</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.11-g0.08</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>227.3766104095246</v>
+        <v>236.3016263737831</v>
       </c>
       <c r="D6" t="n">
-        <v>193.2775777522199</v>
+        <v>202.7478809759036</v>
       </c>
       <c r="E6" t="n">
-        <v>47.60336434187578</v>
+        <v>48.02296538664692</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[316.80331104077624, 508.7905501535252, 219.51133679102156, 371.3828815070573, 581.1229156093686, 587.9257368227724, 570.9783195370366]</t>
+          <t>[301.17774728144036, 494.68729189139236, 197.41309996426264, 344.6047285090625, 562.541226553361, 583.220069313297, 565.9163028453336]</t>
         </is>
       </c>
     </row>
@@ -598,21 +598,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.28-g0.05</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1759.673900235364</v>
+        <v>1758.847872632941</v>
       </c>
       <c r="D7" t="n">
-        <v>1351.032855740508</v>
+        <v>1353.212716638986</v>
       </c>
       <c r="E7" t="n">
-        <v>105.2191632676511</v>
+        <v>105.3519028947413</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[3070.443105642922, 1479.973361908491, 630.7804663095528, 999.0053479070252, 3002.1675989295945, 2035.0564440385149, 1585.652428417881]</t>
+          <t>[3104.9950055760287, 1508.5746594212915, 651.6263691147942, 1010.8207836276775, 3005.864383489536, 2030.4767087204254, 1578.6961156652433]</t>
         </is>
       </c>
     </row>
@@ -624,21 +624,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.22-g0.11</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.21-g0.11</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>283.9996866413552</v>
+        <v>287.8397764802023</v>
       </c>
       <c r="D8" t="n">
-        <v>250.3600261068594</v>
+        <v>254.9296827218318</v>
       </c>
       <c r="E8" t="n">
-        <v>27.59347678905311</v>
+        <v>28.24945219181094</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[380.30851972400274, 386.8808168365863, 947.9508258629836, 1559.4739893367773, 464.1664832916673, 1268.2855123793224, 552.8863463052567]</t>
+          <t>[370.9457761499664, 377.9613558313276, 950.0732090838433, 1559.1953722949227, 459.4136407686226, 1270.1696193019995, 548.2189042881807]</t>
         </is>
       </c>
     </row>
@@ -650,21 +650,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.35-b0.14-g0.05</t>
+          <t>HW-Trend(mul)-seasonal(add)-a0.05-b0.12-g0.05</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>972.9309441467058</v>
+        <v>878.3365195926586</v>
       </c>
       <c r="D9" t="n">
-        <v>696.832413603094</v>
+        <v>599.8484847446723</v>
       </c>
       <c r="E9" t="n">
-        <v>34.65323107458707</v>
+        <v>30.06142121597158</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[4351.614056268247, 4316.351852039614, 0.0, 4570.698566725058, 4057.5515017456037, 3932.3826945113487, 4360.477445735099]</t>
+          <t>[4129.133211467439, 4187.696261567464, 0.0, 4114.548516630495, 3509.5621176496397, 3335.830275106742, 3706.266075390826]</t>
         </is>
       </c>
     </row>
@@ -680,17 +680,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4692.596174553106</v>
+        <v>4813.957411694431</v>
       </c>
       <c r="D10" t="n">
-        <v>3966.583286869793</v>
+        <v>4093.040496737315</v>
       </c>
       <c r="E10" t="n">
-        <v>50.98926954552029</v>
+        <v>52.47407381455725</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[16727.34202541427, 13113.505666532103, 12771.113541106766, 13427.067535160699, 21865.395893661705, 12930.766479015061, 14144.118949411484]</t>
+          <t>[16885.4733154895, 13275.171583829679, 12938.023466181814, 13600.01687921134, 22044.268395268897, 13114.215760936571, 14341.161008607036]</t>
         </is>
       </c>
     </row>
@@ -728,21 +728,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.89-g0.1</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.88-g0.11</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3140.372051758121</v>
+        <v>3154.983149602206</v>
       </c>
       <c r="D12" t="n">
-        <v>2531.199324910177</v>
+        <v>2545.071003704675</v>
       </c>
       <c r="E12" t="n">
-        <v>59.8024405171362</v>
+        <v>64.5144704336559</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[3110.0871807562967, 123.60083887450173, 389.32404120937144, 1335.8989020167262, 2383.6359294397926, 863.228672781997, 386.96357990991146]</t>
+          <t>[3137.36921380645, 33.36718619698968, 337.528996720657, 1318.8465399114145, 2372.6513791725965, 946.9055332940875, 348.96854432491216]</t>
         </is>
       </c>
     </row>
@@ -754,21 +754,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.2-g0.06</t>
+          <t>HW-Trend(mul)-seasonal(mul)-a0.05-b0.2-g0.07</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1764.545580269533</v>
+        <v>1755.044683518549</v>
       </c>
       <c r="D13" t="n">
-        <v>1555.770178221579</v>
+        <v>1545.026039445247</v>
       </c>
       <c r="E13" t="n">
-        <v>36.27568395522115</v>
+        <v>36.12166947119059</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[4085.813868970178, 4836.602677047438, 3246.781715432305, 5096.28263310396, 4387.652822297589, 4136.205207832191, 4332.014111975152]</t>
+          <t>[4117.438099498152, 4853.936859075944, 3256.442380649538, 5109.630986127801, 4373.935614508191, 4143.933829920918, 4334.761157039053]</t>
         </is>
       </c>
     </row>
@@ -780,21 +780,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.59-b0.58-g0.11</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.13-g0.09</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13968.04175366843</v>
+        <v>4176.037148914744</v>
       </c>
       <c r="D14" t="n">
-        <v>13267.11480956027</v>
+        <v>3207.39748491041</v>
       </c>
       <c r="E14" t="n">
-        <v>221.126247476913</v>
+        <v>36.23235315386321</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[16788.9469237623, 11673.282111239849, 16986.195767990957, 23660.922577368183, 27237.406519528187, 27377.365474430375, 29362.43618662148]</t>
+          <t>[9038.138163802907, 2847.9364238274393, 3599.053088576592, 6090.67524527127, 8367.866162765366, 5455.543550863061, 5737.906039800599]</t>
         </is>
       </c>
     </row>
@@ -806,21 +806,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.07-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.06-b0.05-g0.05</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>867.7926320885475</v>
+        <v>848.8057473594365</v>
       </c>
       <c r="D15" t="n">
-        <v>712.2549009247856</v>
+        <v>695.4957867322015</v>
       </c>
       <c r="E15" t="n">
-        <v>40.99804679444166</v>
+        <v>39.80591686797359</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[3209.198959459306, 4301.560199203248, 2307.3166967923753, 4711.068977380947, 7662.202732024307, 2559.5007251821053, 4149.314142245404]</t>
+          <t>[3169.1327708025037, 4263.490672427249, 2271.4624924409245, 4679.760240586072, 7632.021672685023, 2527.763945111393, 4120.253083110792]</t>
         </is>
       </c>
     </row>
@@ -832,21 +832,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.27-g0.18</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.05-g0.23</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1140.10324257694</v>
+        <v>1036.378781269965</v>
       </c>
       <c r="D16" t="n">
-        <v>881.9417432577741</v>
+        <v>837.9773504539256</v>
       </c>
       <c r="E16" t="n">
-        <v>35.39788847152437</v>
+        <v>41.17781511678785</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[3739.0456511104962, 1988.913194014515, 886.6141695131505, 4433.391321402636, 5448.024008105365, 3875.8068058239096, 2531.110315229623]</t>
+          <t>[3847.806826415965, 2149.6794933834085, 1031.7116368800466, 4750.46601959902, 5859.428746329841, 4302.29660156451, 2963.7038557228843]</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1123.967082483953</v>
+        <v>1125.454746087118</v>
       </c>
       <c r="D17" t="n">
-        <v>974.5290236410672</v>
+        <v>972.4308714446685</v>
       </c>
       <c r="E17" t="n">
-        <v>20.40103770904746</v>
+        <v>20.22637371044812</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[4599.7134224892925, 5213.823561728259, 3438.5872082901587, 6328.848437661972, 5955.0096999403995, 2672.001496008873, 6036.8344157721]</t>
+          <t>[4580.131891151981, 5205.527098558593, 3418.405741800323, 6342.287063947331, 5950.782635715397, 2646.0518365848975, 6034.341113911088]</t>
         </is>
       </c>
     </row>
@@ -884,21 +884,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.33-g0.18</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.32-g0.17</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1964.070233266426</v>
+        <v>1937.793480218114</v>
       </c>
       <c r="D18" t="n">
-        <v>1732.536029364453</v>
+        <v>1704.280220166696</v>
       </c>
       <c r="E18" t="n">
-        <v>44.5439851533932</v>
+        <v>43.8882390876235</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[2631.908713553468, 3563.998243748816, 1441.838492994898, 4061.58255038985, 3342.2907138660407, 1907.604308015565, 5837.949184981741]</t>
+          <t>[2683.602687421104, 3581.812576988107, 1516.8518259397274, 4062.296715371269, 3375.8211355255035, 1893.7259830205758, 5729.415124549796]</t>
         </is>
       </c>
     </row>
@@ -910,21 +910,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.09-b0.05-g0.64</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.07-b0.87-g0.05</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>663.5484795499465</v>
+        <v>866.7990019553098</v>
       </c>
       <c r="D19" t="n">
-        <v>603.9988448034521</v>
+        <v>805.1149424630088</v>
       </c>
       <c r="E19" t="n">
-        <v>26.73173758668018</v>
+        <v>36.09890986840371</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[2773.2443579141495, 1823.0179671124645, 851.5299106555732, 1926.0854804303656, 2588.1587316405617, 1491.5651878651302, 2267.2818500317426]</t>
+          <t>[2126.0656923861384, 1753.2384121560701, 876.1567376477565, 1404.5916568618468, 2284.2774743313153, 1343.0967912912272, 994.2861655385294]</t>
         </is>
       </c>
     </row>
@@ -1014,21 +1014,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.56-g0.14</t>
+          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.56-g0.12</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2251.703215383586</v>
+        <v>2368.526731453882</v>
       </c>
       <c r="D23" t="n">
-        <v>1508.831995299819</v>
+        <v>1563.977722519464</v>
       </c>
       <c r="E23" t="n">
-        <v>9.271439447426545</v>
+        <v>9.570442206650863</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[12218.27778572724, 17132.901454933748, 9528.150872531129, 15421.173530997405, 12246.892034079157, 15673.620483486126, 14552.364249658005]</t>
+          <t>[12360.010172443774, 17191.812722378985, 9545.5124953524, 15374.90546515949, 12363.810993033874, 15300.378825496171, 14476.581534410383]</t>
         </is>
       </c>
     </row>
@@ -1040,21 +1040,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.14-b0.37-g0.05</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>677.5235599918963</v>
+        <v>545.8601275461633</v>
       </c>
       <c r="D24" t="n">
-        <v>528.409511341451</v>
+        <v>473.4037760179082</v>
       </c>
       <c r="E24" t="n">
-        <v>15.90141872334303</v>
+        <v>18.41136730520088</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[2556.432099540607, 3284.706231707938, 1467.3869010185547, 3114.400536906187, 2242.1599360691584, 2032.6654823399995, 2453.3822330273983]</t>
+          <t>[2895.23375460418, 3741.6050072421904, 2040.4637019163856, 3804.238925619725, 3054.994370972683, 2999.456837771985, 3536.767936391384]</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.84-b0.21-g0.66</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.14-g0.05</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1485.24487402689</v>
+        <v>1069.552601453288</v>
       </c>
       <c r="D26" t="n">
-        <v>1144.990825185982</v>
+        <v>889.413538090472</v>
       </c>
       <c r="E26" t="n">
-        <v>152.9945412176032</v>
+        <v>102.7334456344538</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[1632.7646932745604, 0.0, 0.0, 0.0, 1391.4992793140732, 793.2263539468155, 0.0]</t>
+          <t>[1307.245894694986, 418.95969389648076, 262.8649254232197, 703.4289402378784, 2131.1769565353375, 1213.8683219579284, 850.5367376212362]</t>
         </is>
       </c>
     </row>
@@ -1118,21 +1118,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.08</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.23-g0.05</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>954.6250362162758</v>
+        <v>984.3865361974417</v>
       </c>
       <c r="D27" t="n">
-        <v>793.161888273081</v>
+        <v>809.1104655793077</v>
       </c>
       <c r="E27" t="n">
-        <v>266.847914863758</v>
+        <v>275.1744457169204</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[1509.1085700966512, 1532.0610623723921, 1409.4255378264445, 2022.161315320735, 1582.1885695108645, 1834.2152136776945, 1615.5037847598087]</t>
+          <t>[1543.1793384885939, 1558.4617758229106, 1507.0135134456748, 2027.0509243776457, 1588.1743879359447, 1873.9105939835806, 1650.7057481666372]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se actualiza ara el SKU 7 la valdiacion de supuestos
</commit_message>
<xml_diff>
--- a/data/output/forecast_results_Recursivo.xlsx
+++ b/data/output/forecast_results_Recursivo.xlsx
@@ -468,21 +468,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.18-g0.26</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.25</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3370.788768434009</v>
+        <v>3274.912277742098</v>
       </c>
       <c r="D2" t="n">
-        <v>2923.907244363023</v>
+        <v>2838.845765118879</v>
       </c>
       <c r="E2" t="n">
-        <v>15.16066528805687</v>
+        <v>14.71100331193007</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[10683.529669664322, 19784.371822121757, 7812.168389276536, 26610.927829068503, 22717.963679664594, 20548.27107161089, 15464.16047229575]</t>
+          <t>[10722.697736602024, 19791.579510256546, 7896.481064513266, 26674.562956476148, 22781.427169962437, 20655.84831741571, 15708.64190945481]</t>
         </is>
       </c>
     </row>
@@ -494,21 +494,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.22-b0.05-g0.16</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.21-b0.05-g0.16</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>323.7320023642358</v>
+        <v>328.3938154364798</v>
       </c>
       <c r="D3" t="n">
-        <v>262.7652561352002</v>
+        <v>268.61976793651</v>
       </c>
       <c r="E3" t="n">
-        <v>19.4951036182859</v>
+        <v>20.00423459076796</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[847.1671447417566, 984.1953725153573, 819.1050615010266, 1335.8387595620368, 1313.4296510772233, 523.171735963137, 1517.7354816930613]</t>
+          <t>[841.7592973951706, 977.8559950696409, 812.5971398487513, 1330.5484574053605, 1308.294050068608, 516.8977418798456, 1511.708942777053]</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>288.9019799464968</v>
+        <v>289.1029541609326</v>
       </c>
       <c r="D4" t="n">
-        <v>251.1698401096004</v>
+        <v>251.0654841691924</v>
       </c>
       <c r="E4" t="n">
-        <v>38.32085397048436</v>
+        <v>38.33089297277512</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[970.3712015611587, 1273.5660968454304, 798.532803654837, 1215.834807565322, 1344.5340265228135, 909.5672696464571, 1561.982921707672]</t>
+          <t>[970.4701112430387, 1272.6144344396685, 799.0775903455095, 1215.3485033485892, 1344.5233960971711, 909.773527265567, 1559.9264875184817]</t>
         </is>
       </c>
     </row>
@@ -572,21 +572,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.11-g0.08</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.07-b0.09-g0.07</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>236.3016263737831</v>
+        <v>227.3766104095246</v>
       </c>
       <c r="D6" t="n">
-        <v>202.7478809759036</v>
+        <v>193.2775777522199</v>
       </c>
       <c r="E6" t="n">
-        <v>48.02296538664692</v>
+        <v>47.60336434187578</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[301.17774728144036, 494.68729189139236, 197.41309996426264, 344.6047285090625, 562.541226553361, 583.220069313297, 565.9163028453336]</t>
+          <t>[316.80331104077624, 508.7905501535252, 219.51133679102156, 371.3828815070573, 581.1229156093686, 587.9257368227724, 570.9783195370366]</t>
         </is>
       </c>
     </row>
@@ -598,21 +598,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.28-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1758.847872632941</v>
+        <v>1759.673900235364</v>
       </c>
       <c r="D7" t="n">
-        <v>1353.212716638986</v>
+        <v>1351.032855740508</v>
       </c>
       <c r="E7" t="n">
-        <v>105.3519028947413</v>
+        <v>105.2191632676511</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[3104.9950055760287, 1508.5746594212915, 651.6263691147942, 1010.8207836276775, 3005.864383489536, 2030.4767087204254, 1578.6961156652433]</t>
+          <t>[3070.443105642922, 1479.973361908491, 630.7804663095528, 999.0053479070252, 3002.1675989295945, 2035.0564440385149, 1585.652428417881]</t>
         </is>
       </c>
     </row>
@@ -624,21 +624,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.21-g0.11</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.22-g0.11</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>287.8397764802023</v>
+        <v>283.9996866413552</v>
       </c>
       <c r="D8" t="n">
-        <v>254.9296827218318</v>
+        <v>250.3600261068594</v>
       </c>
       <c r="E8" t="n">
-        <v>28.24945219181094</v>
+        <v>27.59347678905311</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[370.9457761499664, 377.9613558313276, 950.0732090838433, 1559.1953722949227, 459.4136407686226, 1270.1696193019995, 548.2189042881807]</t>
+          <t>[380.30851972400274, 386.8808168365863, 947.9508258629836, 1559.4739893367773, 464.1664832916673, 1268.2855123793224, 552.8863463052567]</t>
         </is>
       </c>
     </row>
@@ -650,21 +650,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HW-Trend(mul)-seasonal(add)-a0.05-b0.12-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.35-b0.14-g0.05</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>878.3365195926586</v>
+        <v>972.9309441467058</v>
       </c>
       <c r="D9" t="n">
-        <v>599.8484847446723</v>
+        <v>696.832413603094</v>
       </c>
       <c r="E9" t="n">
-        <v>30.06142121597158</v>
+        <v>34.65323107458707</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[4129.133211467439, 4187.696261567464, 0.0, 4114.548516630495, 3509.5621176496397, 3335.830275106742, 3706.266075390826]</t>
+          <t>[4351.614056268247, 4316.351852039614, 0.0, 4570.698566725058, 4057.5515017456037, 3932.3826945113487, 4360.477445735099]</t>
         </is>
       </c>
     </row>
@@ -680,17 +680,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4813.957411694431</v>
+        <v>4692.596174553106</v>
       </c>
       <c r="D10" t="n">
-        <v>4093.040496737315</v>
+        <v>3966.583286869793</v>
       </c>
       <c r="E10" t="n">
-        <v>52.47407381455725</v>
+        <v>50.98926954552029</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[16885.4733154895, 13275.171583829679, 12938.023466181814, 13600.01687921134, 22044.268395268897, 13114.215760936571, 14341.161008607036]</t>
+          <t>[16727.34202541427, 13113.505666532103, 12771.113541106766, 13427.067535160699, 21865.395893661705, 12930.766479015061, 14144.118949411484]</t>
         </is>
       </c>
     </row>
@@ -728,21 +728,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.88-g0.11</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.89-g0.1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3154.983149602206</v>
+        <v>3140.372051758121</v>
       </c>
       <c r="D12" t="n">
-        <v>2545.071003704675</v>
+        <v>2531.199324910177</v>
       </c>
       <c r="E12" t="n">
-        <v>64.5144704336559</v>
+        <v>59.8024405171362</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[3137.36921380645, 33.36718619698968, 337.528996720657, 1318.8465399114145, 2372.6513791725965, 946.9055332940875, 348.96854432491216]</t>
+          <t>[3110.0871807562967, 123.60083887450173, 389.32404120937144, 1335.8989020167262, 2383.6359294397926, 863.228672781997, 386.96357990991146]</t>
         </is>
       </c>
     </row>
@@ -754,21 +754,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HW-Trend(mul)-seasonal(mul)-a0.05-b0.2-g0.07</t>
+          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.2-g0.06</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1755.044683518549</v>
+        <v>1764.545580269533</v>
       </c>
       <c r="D13" t="n">
-        <v>1545.026039445247</v>
+        <v>1555.770178221579</v>
       </c>
       <c r="E13" t="n">
-        <v>36.12166947119059</v>
+        <v>36.27568395522115</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[4117.438099498152, 4853.936859075944, 3256.442380649538, 5109.630986127801, 4373.935614508191, 4143.933829920918, 4334.761157039053]</t>
+          <t>[4085.813868970178, 4836.602677047438, 3246.781715432305, 5096.28263310396, 4387.652822297589, 4136.205207832191, 4332.014111975152]</t>
         </is>
       </c>
     </row>
@@ -780,21 +780,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.13-g0.09</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.59-b0.58-g0.11</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4176.037148914744</v>
+        <v>13968.04175366843</v>
       </c>
       <c r="D14" t="n">
-        <v>3207.39748491041</v>
+        <v>13267.11480956027</v>
       </c>
       <c r="E14" t="n">
-        <v>36.23235315386321</v>
+        <v>221.126247476913</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[9038.138163802907, 2847.9364238274393, 3599.053088576592, 6090.67524527127, 8367.866162765366, 5455.543550863061, 5737.906039800599]</t>
+          <t>[16788.9469237623, 11673.282111239849, 16986.195767990957, 23660.922577368183, 27237.406519528187, 27377.365474430375, 29362.43618662148]</t>
         </is>
       </c>
     </row>
@@ -806,21 +806,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.06-b0.05-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.07-g0.05</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>848.8057473594365</v>
+        <v>867.7926320885475</v>
       </c>
       <c r="D15" t="n">
-        <v>695.4957867322015</v>
+        <v>712.2549009247856</v>
       </c>
       <c r="E15" t="n">
-        <v>39.80591686797359</v>
+        <v>40.99804679444166</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[3169.1327708025037, 4263.490672427249, 2271.4624924409245, 4679.760240586072, 7632.021672685023, 2527.763945111393, 4120.253083110792]</t>
+          <t>[3209.198959459306, 4301.560199203248, 2307.3166967923753, 4711.068977380947, 7662.202732024307, 2559.5007251821053, 4149.314142245404]</t>
         </is>
       </c>
     </row>
@@ -832,21 +832,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.05-g0.23</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.27-g0.18</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1036.378781269965</v>
+        <v>1140.10324257694</v>
       </c>
       <c r="D16" t="n">
-        <v>837.9773504539256</v>
+        <v>881.9417432577741</v>
       </c>
       <c r="E16" t="n">
-        <v>41.17781511678785</v>
+        <v>35.39788847152437</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[3847.806826415965, 2149.6794933834085, 1031.7116368800466, 4750.46601959902, 5859.428746329841, 4302.29660156451, 2963.7038557228843]</t>
+          <t>[3739.0456511104962, 1988.913194014515, 886.6141695131505, 4433.391321402636, 5448.024008105365, 3875.8068058239096, 2531.110315229623]</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1125.454746087118</v>
+        <v>1123.967082483953</v>
       </c>
       <c r="D17" t="n">
-        <v>972.4308714446685</v>
+        <v>974.5290236410672</v>
       </c>
       <c r="E17" t="n">
-        <v>20.22637371044812</v>
+        <v>20.40103770904746</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[4580.131891151981, 5205.527098558593, 3418.405741800323, 6342.287063947331, 5950.782635715397, 2646.0518365848975, 6034.341113911088]</t>
+          <t>[4599.7134224892925, 5213.823561728259, 3438.5872082901587, 6328.848437661972, 5955.0096999403995, 2672.001496008873, 6036.8344157721]</t>
         </is>
       </c>
     </row>
@@ -884,21 +884,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.32-g0.17</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.33-g0.18</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1937.793480218114</v>
+        <v>1964.070233266426</v>
       </c>
       <c r="D18" t="n">
-        <v>1704.280220166696</v>
+        <v>1732.536029364453</v>
       </c>
       <c r="E18" t="n">
-        <v>43.8882390876235</v>
+        <v>44.5439851533932</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[2683.602687421104, 3581.812576988107, 1516.8518259397274, 4062.296715371269, 3375.8211355255035, 1893.7259830205758, 5729.415124549796]</t>
+          <t>[2631.908713553468, 3563.998243748816, 1441.838492994898, 4061.58255038985, 3342.2907138660407, 1907.604308015565, 5837.949184981741]</t>
         </is>
       </c>
     </row>
@@ -910,21 +910,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.07-b0.87-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.09-b0.05-g0.64</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>866.7990019553098</v>
+        <v>663.5484795499465</v>
       </c>
       <c r="D19" t="n">
-        <v>805.1149424630088</v>
+        <v>603.9988448034521</v>
       </c>
       <c r="E19" t="n">
-        <v>36.09890986840371</v>
+        <v>26.73173758668018</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[2126.0656923861384, 1753.2384121560701, 876.1567376477565, 1404.5916568618468, 2284.2774743313153, 1343.0967912912272, 994.2861655385294]</t>
+          <t>[2773.2443579141495, 1823.0179671124645, 851.5299106555732, 1926.0854804303656, 2588.1587316405617, 1491.5651878651302, 2267.2818500317426]</t>
         </is>
       </c>
     </row>
@@ -1014,21 +1014,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.56-g0.12</t>
+          <t>HW-Trend(add)-seasonal(mul)-a0.05-b0.56-g0.14</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2368.526731453882</v>
+        <v>2251.703215383586</v>
       </c>
       <c r="D23" t="n">
-        <v>1563.977722519464</v>
+        <v>1508.831995299819</v>
       </c>
       <c r="E23" t="n">
-        <v>9.570442206650863</v>
+        <v>9.271439447426545</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[12360.010172443774, 17191.812722378985, 9545.5124953524, 15374.90546515949, 12363.810993033874, 15300.378825496171, 14476.581534410383]</t>
+          <t>[12218.27778572724, 17132.901454933748, 9528.150872531129, 15421.173530997405, 12246.892034079157, 15673.620483486126, 14552.364249658005]</t>
         </is>
       </c>
     </row>
@@ -1040,21 +1040,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.14-b0.37-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.05</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>545.8601275461633</v>
+        <v>677.5235599918963</v>
       </c>
       <c r="D24" t="n">
-        <v>473.4037760179082</v>
+        <v>528.409511341451</v>
       </c>
       <c r="E24" t="n">
-        <v>18.41136730520088</v>
+        <v>15.90141872334303</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[2895.23375460418, 3741.6050072421904, 2040.4637019163856, 3804.238925619725, 3054.994370972683, 2999.456837771985, 3536.767936391384]</t>
+          <t>[2556.432099540607, 3284.706231707938, 1467.3869010185547, 3114.400536906187, 2242.1599360691584, 2032.6654823399995, 2453.3822330273983]</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.14-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.84-b0.21-g0.66</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1069.552601453288</v>
+        <v>1485.24487402689</v>
       </c>
       <c r="D26" t="n">
-        <v>889.413538090472</v>
+        <v>1144.990825185982</v>
       </c>
       <c r="E26" t="n">
-        <v>102.7334456344538</v>
+        <v>152.9945412176032</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[1307.245894694986, 418.95969389648076, 262.8649254232197, 703.4289402378784, 2131.1769565353375, 1213.8683219579284, 850.5367376212362]</t>
+          <t>[1632.7646932745604, 0.0, 0.0, 0.0, 1391.4992793140732, 793.2263539468155, 0.0]</t>
         </is>
       </c>
     </row>
@@ -1118,21 +1118,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.23-g0.05</t>
+          <t>HW-Trend(add)-seasonal(add)-a0.05-b0.2-g0.08</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>984.3865361974417</v>
+        <v>954.6250362162758</v>
       </c>
       <c r="D27" t="n">
-        <v>809.1104655793077</v>
+        <v>793.161888273081</v>
       </c>
       <c r="E27" t="n">
-        <v>275.1744457169204</v>
+        <v>266.847914863758</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[1543.1793384885939, 1558.4617758229106, 1507.0135134456748, 2027.0509243776457, 1588.1743879359447, 1873.9105939835806, 1650.7057481666372]</t>
+          <t>[1509.1085700966512, 1532.0610623723921, 1409.4255378264445, 2022.161315320735, 1582.1885695108645, 1834.2152136776945, 1615.5037847598087]</t>
         </is>
       </c>
     </row>

</xml_diff>